<commit_message>
step 4: add file, crustdata, classifier tools and deterministic analysis with tests
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Entire-Checkpoint: 01M4JE6SV45JHZXJSB59W5W7GF
</commit_message>
<xml_diff>
--- a/data/acme/budget_fy27.xlsx
+++ b/data/acme/budget_fy27.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -909,6 +909,106 @@
       </c>
       <c r="O10" t="n">
         <v>3310500</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>headcount</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>84</v>
+      </c>
+      <c r="D11" t="n">
+        <v>85</v>
+      </c>
+      <c r="E11" t="n">
+        <v>85</v>
+      </c>
+      <c r="F11" t="n">
+        <v>86</v>
+      </c>
+      <c r="G11" t="n">
+        <v>86</v>
+      </c>
+      <c r="H11" t="n">
+        <v>87</v>
+      </c>
+      <c r="I11" t="n">
+        <v>87</v>
+      </c>
+      <c r="J11" t="n">
+        <v>88</v>
+      </c>
+      <c r="K11" t="n">
+        <v>88</v>
+      </c>
+      <c r="L11" t="n">
+        <v>89</v>
+      </c>
+      <c r="M11" t="n">
+        <v>89</v>
+      </c>
+      <c r="N11" t="n">
+        <v>90</v>
+      </c>
+      <c r="O11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>people_cost</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>875000</v>
+      </c>
+      <c r="D12" t="n">
+        <v>885417</v>
+      </c>
+      <c r="E12" t="n">
+        <v>885417</v>
+      </c>
+      <c r="F12" t="n">
+        <v>895833</v>
+      </c>
+      <c r="G12" t="n">
+        <v>895833</v>
+      </c>
+      <c r="H12" t="n">
+        <v>906250</v>
+      </c>
+      <c r="I12" t="n">
+        <v>906250</v>
+      </c>
+      <c r="J12" t="n">
+        <v>916667</v>
+      </c>
+      <c r="K12" t="n">
+        <v>916667</v>
+      </c>
+      <c r="L12" t="n">
+        <v>927083</v>
+      </c>
+      <c r="M12" t="n">
+        <v>927083</v>
+      </c>
+      <c r="N12" t="n">
+        <v>937500</v>
+      </c>
+      <c r="O12" t="n">
+        <v>10875000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>